<commit_message>
SQUASHED ONE TINY BUG
.yaml: testing MR24-030-805; reverted pH to offline pH; reverted horizon to 3; mpc_optimizer.py: fixed an issue where Bioreactor.measurement() returns NaNs when there are missing measurements, replaced missing measurements with model predictions; visualize.py: fixed a logical error of calculating RMSEs
</commit_message>
<xml_diff>
--- a/data/mr24-030-038-experiment/MR24-030-038-MasterDataTable.xlsx
+++ b/data/mr24-030-038-experiment/MR24-030-038-MasterDataTable.xlsx
@@ -8,15 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\yl604392\Git\state-space-model\data\mr24-030-038-experiment\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8F4257C9-06BE-49B2-A996-C0EE49E2D1F2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{694197CD-30E1-4CE0-8430-C2C2B92B2F37}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21240" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1170" yWindow="1170" windowWidth="28800" windowHeight="15435" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="2" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$2:$BS$2</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$2:$BS$93</definedName>
   </definedNames>
   <calcPr calcId="191028"/>
   <extLst>
@@ -892,7 +892,7 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -914,6 +914,7 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="22" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="33" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="18" fillId="33" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1295,6 +1296,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A841E7D6-1405-4AC8-A599-0CE4601ECD66}">
+  <sheetPr filterMode="1"/>
   <dimension ref="A1:BS93"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -1360,91 +1362,91 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:71" s="1" customFormat="1" ht="21" x14ac:dyDescent="0.35">
-      <c r="A1" s="10" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="10"/>
-      <c r="C1" s="10"/>
-      <c r="D1" s="10"/>
-      <c r="E1" s="10"/>
-      <c r="F1" s="10"/>
-      <c r="G1" s="11" t="s">
+      <c r="A1" s="11" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="11"/>
+      <c r="C1" s="11"/>
+      <c r="D1" s="11"/>
+      <c r="E1" s="11"/>
+      <c r="F1" s="11"/>
+      <c r="G1" s="12" t="s">
         <v>1</v>
       </c>
-      <c r="H1" s="11"/>
-      <c r="I1" s="11"/>
-      <c r="J1" s="11"/>
-      <c r="K1" s="11"/>
-      <c r="L1" s="11"/>
-      <c r="M1" s="11"/>
-      <c r="N1" s="11"/>
-      <c r="O1" s="11"/>
-      <c r="P1" s="11"/>
-      <c r="Q1" s="11"/>
-      <c r="R1" s="11"/>
-      <c r="S1" s="11"/>
-      <c r="T1" s="11"/>
-      <c r="U1" s="11"/>
-      <c r="V1" s="11"/>
-      <c r="W1" s="11"/>
-      <c r="X1" s="11"/>
-      <c r="Y1" s="11"/>
-      <c r="Z1" s="11"/>
-      <c r="AA1" s="11"/>
-      <c r="AB1" s="11"/>
-      <c r="AC1" s="11"/>
-      <c r="AD1" s="11"/>
-      <c r="AE1" s="11"/>
-      <c r="AF1" s="11"/>
-      <c r="AG1" s="11"/>
-      <c r="AH1" s="12" t="s">
+      <c r="H1" s="12"/>
+      <c r="I1" s="12"/>
+      <c r="J1" s="12"/>
+      <c r="K1" s="12"/>
+      <c r="L1" s="12"/>
+      <c r="M1" s="12"/>
+      <c r="N1" s="12"/>
+      <c r="O1" s="12"/>
+      <c r="P1" s="12"/>
+      <c r="Q1" s="12"/>
+      <c r="R1" s="12"/>
+      <c r="S1" s="12"/>
+      <c r="T1" s="12"/>
+      <c r="U1" s="12"/>
+      <c r="V1" s="12"/>
+      <c r="W1" s="12"/>
+      <c r="X1" s="12"/>
+      <c r="Y1" s="12"/>
+      <c r="Z1" s="12"/>
+      <c r="AA1" s="12"/>
+      <c r="AB1" s="12"/>
+      <c r="AC1" s="12"/>
+      <c r="AD1" s="12"/>
+      <c r="AE1" s="12"/>
+      <c r="AF1" s="12"/>
+      <c r="AG1" s="12"/>
+      <c r="AH1" s="13" t="s">
         <v>2</v>
       </c>
-      <c r="AI1" s="12"/>
-      <c r="AJ1" s="12"/>
-      <c r="AK1" s="12"/>
-      <c r="AL1" s="12"/>
-      <c r="AM1" s="12"/>
-      <c r="AN1" s="12"/>
-      <c r="AO1" s="12"/>
-      <c r="AP1" s="12"/>
-      <c r="AQ1" s="12"/>
-      <c r="AR1" s="12"/>
-      <c r="AS1" s="12"/>
-      <c r="AT1" s="12"/>
-      <c r="AU1" s="12"/>
-      <c r="AV1" s="12"/>
-      <c r="AW1" s="12"/>
-      <c r="AX1" s="13" t="s">
+      <c r="AI1" s="13"/>
+      <c r="AJ1" s="13"/>
+      <c r="AK1" s="13"/>
+      <c r="AL1" s="13"/>
+      <c r="AM1" s="13"/>
+      <c r="AN1" s="13"/>
+      <c r="AO1" s="13"/>
+      <c r="AP1" s="13"/>
+      <c r="AQ1" s="13"/>
+      <c r="AR1" s="13"/>
+      <c r="AS1" s="13"/>
+      <c r="AT1" s="13"/>
+      <c r="AU1" s="13"/>
+      <c r="AV1" s="13"/>
+      <c r="AW1" s="13"/>
+      <c r="AX1" s="14" t="s">
         <v>70</v>
       </c>
-      <c r="AY1" s="13"/>
-      <c r="AZ1" s="13"/>
-      <c r="BA1" s="13"/>
-      <c r="BB1" s="13"/>
-      <c r="BC1" s="14" t="s">
+      <c r="AY1" s="14"/>
+      <c r="AZ1" s="14"/>
+      <c r="BA1" s="14"/>
+      <c r="BB1" s="14"/>
+      <c r="BC1" s="15" t="s">
         <v>64</v>
       </c>
-      <c r="BD1" s="14"/>
-      <c r="BE1" s="14"/>
-      <c r="BF1" s="15" t="s">
+      <c r="BD1" s="15"/>
+      <c r="BE1" s="15"/>
+      <c r="BF1" s="16" t="s">
         <v>62</v>
       </c>
-      <c r="BG1" s="15"/>
-      <c r="BH1" s="15"/>
-      <c r="BI1" s="15"/>
-      <c r="BJ1" s="15"/>
-      <c r="BK1" s="15"/>
-      <c r="BL1" s="15"/>
-      <c r="BM1" s="15"/>
-      <c r="BN1" s="15"/>
-      <c r="BO1" s="15"/>
-      <c r="BP1" s="15"/>
-      <c r="BQ1" s="9" t="s">
+      <c r="BG1" s="16"/>
+      <c r="BH1" s="16"/>
+      <c r="BI1" s="16"/>
+      <c r="BJ1" s="16"/>
+      <c r="BK1" s="16"/>
+      <c r="BL1" s="16"/>
+      <c r="BM1" s="16"/>
+      <c r="BN1" s="16"/>
+      <c r="BO1" s="16"/>
+      <c r="BP1" s="16"/>
+      <c r="BQ1" s="10" t="s">
         <v>66</v>
       </c>
-      <c r="BR1" s="9"/>
-      <c r="BS1" s="9"/>
+      <c r="BR1" s="10"/>
+      <c r="BS1" s="10"/>
     </row>
     <row r="2" spans="1:71" s="1" customFormat="1" ht="60" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
@@ -1661,7 +1663,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="3" spans="1:71" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:71" hidden="1" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>53</v>
       </c>
@@ -1849,7 +1851,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:71" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:71" hidden="1" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>54</v>
       </c>
@@ -2040,7 +2042,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:71" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:71" hidden="1" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>55</v>
       </c>
@@ -2231,7 +2233,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:71" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:71" hidden="1" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>56</v>
       </c>
@@ -2613,7 +2615,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:71" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:71" hidden="1" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>58</v>
       </c>
@@ -2807,7 +2809,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:71" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:71" hidden="1" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>53</v>
       </c>
@@ -2995,7 +2997,7 @@
         <v>17.4800465</v>
       </c>
     </row>
-    <row r="10" spans="1:71" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:71" hidden="1" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>54</v>
       </c>
@@ -3186,7 +3188,7 @@
         <v>17.745815000000004</v>
       </c>
     </row>
-    <row r="11" spans="1:71" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:71" hidden="1" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>55</v>
       </c>
@@ -3377,7 +3379,7 @@
         <v>17.393346000000001</v>
       </c>
     </row>
-    <row r="12" spans="1:71" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:71" hidden="1" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>56</v>
       </c>
@@ -3759,7 +3761,7 @@
         <v>14.022246000000001</v>
       </c>
     </row>
-    <row r="14" spans="1:71" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:71" hidden="1" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>58</v>
       </c>
@@ -3953,7 +3955,7 @@
         <v>17.715888</v>
       </c>
     </row>
-    <row r="15" spans="1:71" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:71" hidden="1" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>53</v>
       </c>
@@ -4141,7 +4143,7 @@
         <v>11.539479000000002</v>
       </c>
     </row>
-    <row r="16" spans="1:71" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:71" hidden="1" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>54</v>
       </c>
@@ -4332,7 +4334,7 @@
         <v>12.608789925000002</v>
       </c>
     </row>
-    <row r="17" spans="1:71" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:71" hidden="1" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>55</v>
       </c>
@@ -4523,7 +4525,7 @@
         <v>11.993802225000001</v>
       </c>
     </row>
-    <row r="18" spans="1:71" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:71" hidden="1" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>56</v>
       </c>
@@ -4887,7 +4889,7 @@
         <v>3.9633683594627347</v>
       </c>
     </row>
-    <row r="20" spans="1:71" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:71" hidden="1" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>58</v>
       </c>
@@ -5081,7 +5083,7 @@
         <v>8.4828514616618094</v>
       </c>
     </row>
-    <row r="21" spans="1:71" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:71" hidden="1" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>53</v>
       </c>
@@ -5269,7 +5271,7 @@
         <v>13.18215</v>
       </c>
     </row>
-    <row r="22" spans="1:71" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:71" hidden="1" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>54</v>
       </c>
@@ -5460,7 +5462,7 @@
         <v>13.150274999999999</v>
       </c>
     </row>
-    <row r="23" spans="1:71" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:71" hidden="1" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>55</v>
       </c>
@@ -5845,7 +5847,7 @@
         <v>5.3590759753051112</v>
       </c>
     </row>
-    <row r="25" spans="1:71" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:71" hidden="1" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>58</v>
       </c>
@@ -6039,7 +6041,7 @@
         <v>7.4775654747660001</v>
       </c>
     </row>
-    <row r="26" spans="1:71" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:71" hidden="1" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>53</v>
       </c>
@@ -6227,7 +6229,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="27" spans="1:71" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:71" hidden="1" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>54</v>
       </c>
@@ -6418,7 +6420,7 @@
         <v>6.7380460000000006</v>
       </c>
     </row>
-    <row r="28" spans="1:71" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:71" hidden="1" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>55</v>
       </c>
@@ -6652,9 +6654,7 @@
       <c r="P29">
         <v>16.8</v>
       </c>
-      <c r="Q29">
-        <v>0</v>
-      </c>
+      <c r="Q29" s="9"/>
       <c r="R29">
         <v>1.33</v>
       </c>
@@ -6800,7 +6800,7 @@
         <v>4.2185063447336155</v>
       </c>
     </row>
-    <row r="30" spans="1:71" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:71" hidden="1" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
         <v>58</v>
       </c>
@@ -6991,7 +6991,7 @@
         <v>3.6766410485124208</v>
       </c>
     </row>
-    <row r="31" spans="1:71" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:71" hidden="1" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
         <v>53</v>
       </c>
@@ -7179,7 +7179,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="32" spans="1:71" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:71" hidden="1" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
         <v>54</v>
       </c>
@@ -7370,7 +7370,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="33" spans="1:71" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:71" hidden="1" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
         <v>55</v>
       </c>
@@ -7755,7 +7755,7 @@
         <v>7.6791147043425241</v>
       </c>
     </row>
-    <row r="35" spans="1:71" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:71" hidden="1" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
         <v>58</v>
       </c>
@@ -7949,7 +7949,7 @@
         <v>10.261394893996174</v>
       </c>
     </row>
-    <row r="36" spans="1:71" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:71" hidden="1" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
         <v>53</v>
       </c>
@@ -8134,7 +8134,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="37" spans="1:71" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:71" hidden="1" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
         <v>54</v>
       </c>
@@ -8322,7 +8322,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="38" spans="1:71" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:71" hidden="1" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
         <v>55</v>
       </c>
@@ -8698,7 +8698,7 @@
         <v>8.4915585188980369</v>
       </c>
     </row>
-    <row r="40" spans="1:71" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:71" hidden="1" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
         <v>58</v>
       </c>
@@ -8889,7 +8889,7 @@
         <v>2.3220682771976411</v>
       </c>
     </row>
-    <row r="41" spans="1:71" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:71" hidden="1" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
         <v>53</v>
       </c>
@@ -9074,7 +9074,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="42" spans="1:71" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:71" hidden="1" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
         <v>54</v>
       </c>
@@ -9262,7 +9262,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="43" spans="1:71" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:71" hidden="1" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
         <v>55</v>
       </c>
@@ -9641,7 +9641,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="45" spans="1:71" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:71" hidden="1" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
         <v>58</v>
       </c>
@@ -9832,7 +9832,7 @@
         <v>3.0977345708595014</v>
       </c>
     </row>
-    <row r="46" spans="1:71" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:71" hidden="1" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
         <v>53</v>
       </c>
@@ -10014,7 +10014,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="47" spans="1:71" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:71" hidden="1" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
         <v>54</v>
       </c>
@@ -10199,7 +10199,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="48" spans="1:71" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:71" hidden="1" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
         <v>55</v>
       </c>
@@ -10424,9 +10424,7 @@
       <c r="P49">
         <v>17.399999999999999</v>
       </c>
-      <c r="Q49">
-        <v>0</v>
-      </c>
+      <c r="Q49" s="9"/>
       <c r="R49">
         <v>1.8</v>
       </c>
@@ -10572,7 +10570,7 @@
         <v>6.6672711206767126</v>
       </c>
     </row>
-    <row r="50" spans="1:71" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:71" hidden="1" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
         <v>58</v>
       </c>
@@ -10760,7 +10758,7 @@
         <v>6.8219871831206671</v>
       </c>
     </row>
-    <row r="51" spans="1:71" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:71" hidden="1" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
         <v>53</v>
       </c>
@@ -10945,7 +10943,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="52" spans="1:71" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:71" hidden="1" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
         <v>54</v>
       </c>
@@ -11133,7 +11131,7 @@
         <v>14.179864050000001</v>
       </c>
     </row>
-    <row r="53" spans="1:71" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:71" hidden="1" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
         <v>55</v>
       </c>
@@ -11512,7 +11510,7 @@
         <v>1.2053112985361027</v>
       </c>
     </row>
-    <row r="55" spans="1:71" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:71" hidden="1" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
         <v>58</v>
       </c>
@@ -11703,7 +11701,7 @@
         <v>5.7991313075208026</v>
       </c>
     </row>
-    <row r="56" spans="1:71" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:71" hidden="1" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
         <v>53</v>
       </c>
@@ -11888,7 +11886,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="57" spans="1:71" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:71" hidden="1" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
         <v>54</v>
       </c>
@@ -12076,7 +12074,7 @@
         <v>12.103236375000002</v>
       </c>
     </row>
-    <row r="58" spans="1:71" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:71" hidden="1" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
         <v>55</v>
       </c>
@@ -12455,7 +12453,7 @@
         <v>6.9891921680878912</v>
       </c>
     </row>
-    <row r="60" spans="1:71" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:71" hidden="1" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
         <v>58</v>
       </c>
@@ -12646,7 +12644,7 @@
         <v>7.1864023795214536</v>
       </c>
     </row>
-    <row r="61" spans="1:71" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:71" hidden="1" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
         <v>53</v>
       </c>
@@ -12831,7 +12829,7 @@
         <v>9.7536480000000001</v>
       </c>
     </row>
-    <row r="62" spans="1:71" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:71" hidden="1" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
         <v>54</v>
       </c>
@@ -13019,7 +13017,7 @@
         <v>11.520405</v>
       </c>
     </row>
-    <row r="63" spans="1:71" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:71" hidden="1" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
         <v>55</v>
       </c>
@@ -13250,6 +13248,7 @@
       <c r="P64">
         <v>17.2</v>
       </c>
+      <c r="Q64" s="9"/>
       <c r="R64">
         <v>3.99</v>
       </c>
@@ -13395,7 +13394,7 @@
         <v>5.8497357969925208</v>
       </c>
     </row>
-    <row r="65" spans="1:71" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:71" hidden="1" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
         <v>58</v>
       </c>
@@ -13586,7 +13585,7 @@
         <v>1.9961199999999997E-4</v>
       </c>
     </row>
-    <row r="66" spans="1:71" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:71" hidden="1" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
         <v>53</v>
       </c>
@@ -13768,7 +13767,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="67" spans="1:71" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:71" hidden="1" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
         <v>54</v>
       </c>
@@ -13950,7 +13949,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="68" spans="1:71" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:71" hidden="1" x14ac:dyDescent="0.25">
       <c r="A68" t="s">
         <v>55</v>
       </c>
@@ -14314,7 +14313,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="70" spans="1:71" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:71" hidden="1" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
         <v>58</v>
       </c>
@@ -14496,7 +14495,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="71" spans="1:71" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:71" hidden="1" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
         <v>84</v>
       </c>
@@ -14696,7 +14695,7 @@
         <v>1.685E-4</v>
       </c>
     </row>
-    <row r="72" spans="1:71" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:71" hidden="1" x14ac:dyDescent="0.25">
       <c r="A72" t="s">
         <v>85</v>
       </c>
@@ -14896,7 +14895,7 @@
         <v>1.685E-4</v>
       </c>
     </row>
-    <row r="73" spans="1:71" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:71" hidden="1" x14ac:dyDescent="0.25">
       <c r="A73" t="s">
         <v>86</v>
       </c>
@@ -15096,7 +15095,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="74" spans="1:71" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:71" hidden="1" x14ac:dyDescent="0.25">
       <c r="A74" t="s">
         <v>87</v>
       </c>
@@ -15296,7 +15295,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="75" spans="1:71" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:71" hidden="1" x14ac:dyDescent="0.25">
       <c r="A75" t="s">
         <v>84</v>
       </c>
@@ -15499,7 +15498,7 @@
         <v>16.832071720300799</v>
       </c>
     </row>
-    <row r="76" spans="1:71" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:71" hidden="1" x14ac:dyDescent="0.25">
       <c r="A76" t="s">
         <v>85</v>
       </c>
@@ -15705,7 +15704,7 @@
         <v>18.617318338672099</v>
       </c>
     </row>
-    <row r="77" spans="1:71" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:71" hidden="1" x14ac:dyDescent="0.25">
       <c r="A77" t="s">
         <v>86</v>
       </c>
@@ -15905,7 +15904,7 @@
         <v>16.512855499999997</v>
       </c>
     </row>
-    <row r="78" spans="1:71" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:71" hidden="1" x14ac:dyDescent="0.25">
       <c r="A78" t="s">
         <v>87</v>
       </c>
@@ -16105,7 +16104,7 @@
         <v>17.037286999999999</v>
       </c>
     </row>
-    <row r="79" spans="1:71" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:71" hidden="1" x14ac:dyDescent="0.25">
       <c r="A79" t="s">
         <v>84</v>
       </c>
@@ -16311,7 +16310,7 @@
         <v>12.1026345792793</v>
       </c>
     </row>
-    <row r="80" spans="1:71" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:71" hidden="1" x14ac:dyDescent="0.25">
       <c r="A80" t="s">
         <v>86</v>
       </c>
@@ -16514,7 +16513,7 @@
         <v>12.887707500000001</v>
       </c>
     </row>
-    <row r="81" spans="1:71" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:71" hidden="1" x14ac:dyDescent="0.25">
       <c r="A81" t="s">
         <v>87</v>
       </c>
@@ -16717,7 +16716,7 @@
         <v>10.962813374999998</v>
       </c>
     </row>
-    <row r="82" spans="1:71" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:71" hidden="1" x14ac:dyDescent="0.25">
       <c r="A82" t="s">
         <v>84</v>
       </c>
@@ -16920,7 +16919,7 @@
         <v>11.3869050015914</v>
       </c>
     </row>
-    <row r="83" spans="1:71" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:71" hidden="1" x14ac:dyDescent="0.25">
       <c r="A83" t="s">
         <v>86</v>
       </c>
@@ -17120,7 +17119,7 @@
         <v>13.070538324999999</v>
       </c>
     </row>
-    <row r="84" spans="1:71" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:71" hidden="1" x14ac:dyDescent="0.25">
       <c r="A84" t="s">
         <v>84</v>
       </c>
@@ -17329,7 +17328,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="85" spans="1:71" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:71" hidden="1" x14ac:dyDescent="0.25">
       <c r="A85" t="s">
         <v>86</v>
       </c>
@@ -17496,7 +17495,7 @@
         <v>7.4749999999999996</v>
       </c>
     </row>
-    <row r="86" spans="1:71" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:71" hidden="1" x14ac:dyDescent="0.25">
       <c r="A86" t="s">
         <v>84</v>
       </c>
@@ -17702,7 +17701,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="87" spans="1:71" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:71" hidden="1" x14ac:dyDescent="0.25">
       <c r="A87" t="s">
         <v>84</v>
       </c>
@@ -17908,7 +17907,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="88" spans="1:71" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:71" hidden="1" x14ac:dyDescent="0.25">
       <c r="A88" t="s">
         <v>84</v>
       </c>
@@ -18114,7 +18113,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="89" spans="1:71" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:71" hidden="1" x14ac:dyDescent="0.25">
       <c r="A89" t="s">
         <v>84</v>
       </c>
@@ -18320,7 +18319,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="90" spans="1:71" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:71" hidden="1" x14ac:dyDescent="0.25">
       <c r="A90" t="s">
         <v>84</v>
       </c>
@@ -18523,7 +18522,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="91" spans="1:71" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:71" hidden="1" x14ac:dyDescent="0.25">
       <c r="A91" t="s">
         <v>84</v>
       </c>
@@ -18729,7 +18728,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="92" spans="1:71" x14ac:dyDescent="0.25">
+    <row r="92" spans="1:71" hidden="1" x14ac:dyDescent="0.25">
       <c r="A92" t="s">
         <v>84</v>
       </c>
@@ -18932,7 +18931,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="93" spans="1:71" x14ac:dyDescent="0.25">
+    <row r="93" spans="1:71" hidden="1" x14ac:dyDescent="0.25">
       <c r="A93" t="s">
         <v>84</v>
       </c>
@@ -19127,7 +19126,13 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A2:BS2" xr:uid="{A841E7D6-1405-4AC8-A599-0CE4601ECD66}"/>
+  <autoFilter ref="A2:BS93" xr:uid="{A841E7D6-1405-4AC8-A599-0CE4601ECD66}">
+    <filterColumn colId="0">
+      <filters>
+        <filter val="MR24-030-805"/>
+      </filters>
+    </filterColumn>
+  </autoFilter>
   <mergeCells count="7">
     <mergeCell ref="BQ1:BS1"/>
     <mergeCell ref="A1:F1"/>
@@ -19143,12 +19148,21 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="a198008e-c7f6-4ed0-9865-26ace3c97b59" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="34d8c884-fe7e-4d4f-a833-b92a2823f74b">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <SharedWithUsers xmlns="a198008e-c7f6-4ed0-9865-26ace3c97b59">
+      <UserInfo>
+        <DisplayName/>
+        <AccountId xsi:nil="true"/>
+        <AccountType/>
+      </UserInfo>
+    </SharedWithUsers>
+  </documentManagement>
+</p:properties>
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -19375,27 +19389,27 @@
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="a198008e-c7f6-4ed0-9865-26ace3c97b59" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="34d8c884-fe7e-4d4f-a833-b92a2823f74b">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <SharedWithUsers xmlns="a198008e-c7f6-4ed0-9865-26ace3c97b59">
-      <UserInfo>
-        <DisplayName/>
-        <AccountId xsi:nil="true"/>
-        <AccountType/>
-      </UserInfo>
-    </SharedWithUsers>
-  </documentManagement>
-</p:properties>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6FA2C79D-5C43-4F8C-8CB2-6CBFC4591548}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{81736866-79EE-4C47-B374-7C3565856A36}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="34d8c884-fe7e-4d4f-a833-b92a2823f74b"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="a198008e-c7f6-4ed0-9865-26ace3c97b59"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -19420,18 +19434,9 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{81736866-79EE-4C47-B374-7C3565856A36}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6FA2C79D-5C43-4F8C-8CB2-6CBFC4591548}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="34d8c884-fe7e-4d4f-a833-b92a2823f74b"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="a198008e-c7f6-4ed0-9865-26ace3c97b59"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>